<commit_message>
Update README, Docker, PM2 config and screenshots for the universal Smart MIS
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xykczr9N564ruTLrBqtJzY
</commit_message>
<xml_diff>
--- a/samples/hr-employees.xlsx
+++ b/samples/hr-employees.xlsx
@@ -455,7 +455,7 @@
         <v>24</v>
       </c>
       <c r="G2" s="1" t="d">
-        <v>2020-12-08T05:30:00.000Z</v>
+        <v>2020-12-08T00:00:00.000Z</v>
       </c>
       <c r="H2">
         <v>47300</v>
@@ -490,7 +490,7 @@
         <v>23</v>
       </c>
       <c r="G3" s="1" t="d">
-        <v>2016-12-11T05:30:00.000Z</v>
+        <v>2016-12-11T00:00:00.000Z</v>
       </c>
       <c r="H3">
         <v>79500</v>
@@ -525,7 +525,7 @@
         <v>35</v>
       </c>
       <c r="G4" s="1" t="d">
-        <v>2016-10-07T05:30:00.000Z</v>
+        <v>2016-10-07T00:00:00.000Z</v>
       </c>
       <c r="H4">
         <v>84700</v>
@@ -560,7 +560,7 @@
         <v>41</v>
       </c>
       <c r="G5" s="1" t="d">
-        <v>2021-09-01T05:30:00.000Z</v>
+        <v>2021-09-01T00:00:00.000Z</v>
       </c>
       <c r="H5">
         <v>100000</v>
@@ -595,7 +595,7 @@
         <v>55</v>
       </c>
       <c r="G6" s="1" t="d">
-        <v>2022-04-12T05:30:00.000Z</v>
+        <v>2022-04-12T00:00:00.000Z</v>
       </c>
       <c r="H6">
         <v>125600</v>
@@ -630,7 +630,7 @@
         <v>22</v>
       </c>
       <c r="G7" s="1" t="d">
-        <v>2017-06-10T05:30:00.000Z</v>
+        <v>2017-06-10T00:00:00.000Z</v>
       </c>
       <c r="H7">
         <v>73600</v>
@@ -665,7 +665,7 @@
         <v>55</v>
       </c>
       <c r="G8" s="1" t="d">
-        <v>2023-05-12T05:30:00.000Z</v>
+        <v>2023-05-12T00:00:00.000Z</v>
       </c>
       <c r="H8">
         <v>39500</v>
@@ -700,7 +700,7 @@
         <v>40</v>
       </c>
       <c r="G9" s="1" t="d">
-        <v>2021-04-22T05:30:00.000Z</v>
+        <v>2021-04-22T00:00:00.000Z</v>
       </c>
       <c r="H9">
         <v>98800</v>
@@ -735,7 +735,7 @@
         <v>23</v>
       </c>
       <c r="G10" s="1" t="d">
-        <v>2025-11-06T05:30:00.000Z</v>
+        <v>2025-11-06T00:00:00.000Z</v>
       </c>
       <c r="H10">
         <v>60500</v>
@@ -770,7 +770,7 @@
         <v>57</v>
       </c>
       <c r="G11" s="1" t="d">
-        <v>2021-12-06T05:30:00.000Z</v>
+        <v>2021-12-06T00:00:00.000Z</v>
       </c>
       <c r="H11">
         <v>73500</v>
@@ -805,7 +805,7 @@
         <v>44</v>
       </c>
       <c r="G12" s="1" t="d">
-        <v>2022-11-01T05:30:00.000Z</v>
+        <v>2022-11-01T00:00:00.000Z</v>
       </c>
       <c r="H12">
         <v>88400</v>
@@ -840,7 +840,7 @@
         <v>30</v>
       </c>
       <c r="G13" s="1" t="d">
-        <v>2018-12-19T05:30:00.000Z</v>
+        <v>2018-12-19T00:00:00.000Z</v>
       </c>
       <c r="H13">
         <v>81000</v>
@@ -875,7 +875,7 @@
         <v>53</v>
       </c>
       <c r="G14" s="1" t="d">
-        <v>2022-09-01T05:30:00.000Z</v>
+        <v>2022-09-01T00:00:00.000Z</v>
       </c>
       <c r="H14">
         <v>54200</v>
@@ -910,7 +910,7 @@
         <v>33</v>
       </c>
       <c r="G15" s="1" t="d">
-        <v>2018-03-05T05:30:00.000Z</v>
+        <v>2018-03-05T00:00:00.000Z</v>
       </c>
       <c r="H15">
         <v>72100</v>
@@ -945,7 +945,7 @@
         <v>42</v>
       </c>
       <c r="G16" s="1" t="d">
-        <v>2019-03-11T05:30:00.000Z</v>
+        <v>2019-03-11T00:00:00.000Z</v>
       </c>
       <c r="H16">
         <v>45700</v>
@@ -980,7 +980,7 @@
         <v>50</v>
       </c>
       <c r="G17" s="1" t="d">
-        <v>2024-02-16T05:30:00.000Z</v>
+        <v>2024-02-16T00:00:00.000Z</v>
       </c>
       <c r="H17">
         <v>57800</v>
@@ -1015,7 +1015,7 @@
         <v>36</v>
       </c>
       <c r="G18" s="1" t="d">
-        <v>2019-09-27T05:30:00.000Z</v>
+        <v>2019-09-27T00:00:00.000Z</v>
       </c>
       <c r="H18">
         <v>121700</v>
@@ -1050,7 +1050,7 @@
         <v>49</v>
       </c>
       <c r="G19" s="1" t="d">
-        <v>2025-10-17T05:30:00.000Z</v>
+        <v>2025-10-17T00:00:00.000Z</v>
       </c>
       <c r="H19">
         <v>51200</v>
@@ -1085,7 +1085,7 @@
         <v>24</v>
       </c>
       <c r="G20" s="1" t="d">
-        <v>2017-06-11T05:30:00.000Z</v>
+        <v>2017-06-11T00:00:00.000Z</v>
       </c>
       <c r="H20">
         <v>43400</v>
@@ -1120,7 +1120,7 @@
         <v>51</v>
       </c>
       <c r="G21" s="1" t="d">
-        <v>2020-03-05T05:30:00.000Z</v>
+        <v>2020-03-05T00:00:00.000Z</v>
       </c>
       <c r="H21">
         <v>74900</v>
@@ -1155,7 +1155,7 @@
         <v>27</v>
       </c>
       <c r="G22" s="1" t="d">
-        <v>2018-06-12T05:30:00.000Z</v>
+        <v>2018-06-12T00:00:00.000Z</v>
       </c>
       <c r="H22">
         <v>110300</v>
@@ -1190,7 +1190,7 @@
         <v>51</v>
       </c>
       <c r="G23" s="1" t="d">
-        <v>2016-12-15T05:30:00.000Z</v>
+        <v>2016-12-15T00:00:00.000Z</v>
       </c>
       <c r="H23">
         <v>52600</v>
@@ -1225,7 +1225,7 @@
         <v>49</v>
       </c>
       <c r="G24" s="1" t="d">
-        <v>2020-12-26T05:30:00.000Z</v>
+        <v>2020-12-26T00:00:00.000Z</v>
       </c>
       <c r="H24">
         <v>35800</v>
@@ -1260,7 +1260,7 @@
         <v>48</v>
       </c>
       <c r="G25" s="1" t="d">
-        <v>2024-01-20T05:30:00.000Z</v>
+        <v>2024-01-20T00:00:00.000Z</v>
       </c>
       <c r="H25">
         <v>79000</v>
@@ -1295,7 +1295,7 @@
         <v>31</v>
       </c>
       <c r="G26" s="1" t="d">
-        <v>2019-03-22T05:30:00.000Z</v>
+        <v>2019-03-22T00:00:00.000Z</v>
       </c>
       <c r="H26">
         <v>53800</v>
@@ -1330,7 +1330,7 @@
         <v>56</v>
       </c>
       <c r="G27" s="1" t="d">
-        <v>2023-07-09T05:30:00.000Z</v>
+        <v>2023-07-09T00:00:00.000Z</v>
       </c>
       <c r="H27">
         <v>43700</v>
@@ -1365,7 +1365,7 @@
         <v>55</v>
       </c>
       <c r="G28" s="1" t="d">
-        <v>2016-04-24T05:30:00.000Z</v>
+        <v>2016-04-24T00:00:00.000Z</v>
       </c>
       <c r="H28">
         <v>64500</v>
@@ -1400,7 +1400,7 @@
         <v>37</v>
       </c>
       <c r="G29" s="1" t="d">
-        <v>2016-08-06T05:30:00.000Z</v>
+        <v>2016-08-06T00:00:00.000Z</v>
       </c>
       <c r="H29">
         <v>61500</v>
@@ -1435,7 +1435,7 @@
         <v>36</v>
       </c>
       <c r="G30" s="1" t="d">
-        <v>2024-08-12T05:30:00.000Z</v>
+        <v>2024-08-12T00:00:00.000Z</v>
       </c>
       <c r="H30">
         <v>48200</v>
@@ -1470,7 +1470,7 @@
         <v>35</v>
       </c>
       <c r="G31" s="1" t="d">
-        <v>2021-04-12T05:30:00.000Z</v>
+        <v>2021-04-12T00:00:00.000Z</v>
       </c>
       <c r="H31">
         <v>53000</v>
@@ -1505,7 +1505,7 @@
         <v>54</v>
       </c>
       <c r="G32" s="1" t="d">
-        <v>2017-12-12T05:30:00.000Z</v>
+        <v>2017-12-12T00:00:00.000Z</v>
       </c>
       <c r="H32">
         <v>94700</v>
@@ -1540,7 +1540,7 @@
         <v>23</v>
       </c>
       <c r="G33" s="1" t="d">
-        <v>2018-04-20T05:30:00.000Z</v>
+        <v>2018-04-20T00:00:00.000Z</v>
       </c>
       <c r="H33">
         <v>44700</v>
@@ -1575,7 +1575,7 @@
         <v>26</v>
       </c>
       <c r="G34" s="1" t="d">
-        <v>2016-08-21T05:30:00.000Z</v>
+        <v>2016-08-21T00:00:00.000Z</v>
       </c>
       <c r="H34">
         <v>45800</v>
@@ -1610,7 +1610,7 @@
         <v>57</v>
       </c>
       <c r="G35" s="1" t="d">
-        <v>2024-11-07T05:30:00.000Z</v>
+        <v>2024-11-07T00:00:00.000Z</v>
       </c>
       <c r="H35">
         <v>72900</v>
@@ -1645,7 +1645,7 @@
         <v>43</v>
       </c>
       <c r="G36" s="1" t="d">
-        <v>2024-02-09T05:30:00.000Z</v>
+        <v>2024-02-09T00:00:00.000Z</v>
       </c>
       <c r="H36">
         <v>56700</v>
@@ -1680,7 +1680,7 @@
         <v>23</v>
       </c>
       <c r="G37" s="1" t="d">
-        <v>2017-11-02T05:30:00.000Z</v>
+        <v>2017-11-02T00:00:00.000Z</v>
       </c>
       <c r="H37">
         <v>65600</v>
@@ -1715,7 +1715,7 @@
         <v>36</v>
       </c>
       <c r="G38" s="1" t="d">
-        <v>2023-04-26T05:30:00.000Z</v>
+        <v>2023-04-26T00:00:00.000Z</v>
       </c>
       <c r="H38">
         <v>64500</v>
@@ -1750,7 +1750,7 @@
         <v>44</v>
       </c>
       <c r="G39" s="1" t="d">
-        <v>2022-04-12T05:30:00.000Z</v>
+        <v>2022-04-12T00:00:00.000Z</v>
       </c>
       <c r="H39">
         <v>93300</v>
@@ -1785,7 +1785,7 @@
         <v>37</v>
       </c>
       <c r="G40" s="1" t="d">
-        <v>2023-01-02T05:30:00.000Z</v>
+        <v>2023-01-02T00:00:00.000Z</v>
       </c>
       <c r="H40">
         <v>76000</v>
@@ -1820,7 +1820,7 @@
         <v>53</v>
       </c>
       <c r="G41" s="1" t="d">
-        <v>2021-05-05T05:30:00.000Z</v>
+        <v>2021-05-05T00:00:00.000Z</v>
       </c>
       <c r="H41">
         <v>45200</v>
@@ -1855,7 +1855,7 @@
         <v>55</v>
       </c>
       <c r="G42" s="1" t="d">
-        <v>2017-09-21T05:30:00.000Z</v>
+        <v>2017-09-21T00:00:00.000Z</v>
       </c>
       <c r="H42">
         <v>62900</v>
@@ -1890,7 +1890,7 @@
         <v>40</v>
       </c>
       <c r="G43" s="1" t="d">
-        <v>2023-10-22T05:30:00.000Z</v>
+        <v>2023-10-22T00:00:00.000Z</v>
       </c>
       <c r="H43">
         <v>45400</v>
@@ -1925,7 +1925,7 @@
         <v>24</v>
       </c>
       <c r="G44" s="1" t="d">
-        <v>2022-10-11T05:30:00.000Z</v>
+        <v>2022-10-11T00:00:00.000Z</v>
       </c>
       <c r="H44">
         <v>64900</v>
@@ -1960,7 +1960,7 @@
         <v>27</v>
       </c>
       <c r="G45" s="1" t="d">
-        <v>2024-09-20T05:30:00.000Z</v>
+        <v>2024-09-20T00:00:00.000Z</v>
       </c>
       <c r="H45">
         <v>80500</v>
@@ -1995,7 +1995,7 @@
         <v>26</v>
       </c>
       <c r="G46" s="1" t="d">
-        <v>2025-07-03T05:30:00.000Z</v>
+        <v>2025-07-03T00:00:00.000Z</v>
       </c>
       <c r="H46">
         <v>113900</v>
@@ -2030,7 +2030,7 @@
         <v>54</v>
       </c>
       <c r="G47" s="1" t="d">
-        <v>2022-08-09T05:30:00.000Z</v>
+        <v>2022-08-09T00:00:00.000Z</v>
       </c>
       <c r="H47">
         <v>59100</v>
@@ -2065,7 +2065,7 @@
         <v>37</v>
       </c>
       <c r="G48" s="1" t="d">
-        <v>2024-05-27T05:30:00.000Z</v>
+        <v>2024-05-27T00:00:00.000Z</v>
       </c>
       <c r="H48">
         <v>49800</v>
@@ -2100,7 +2100,7 @@
         <v>39</v>
       </c>
       <c r="G49" s="1" t="d">
-        <v>2025-02-04T05:30:00.000Z</v>
+        <v>2025-02-04T00:00:00.000Z</v>
       </c>
       <c r="H49">
         <v>58500</v>
@@ -2135,7 +2135,7 @@
         <v>34</v>
       </c>
       <c r="G50" s="1" t="d">
-        <v>2022-05-08T05:30:00.000Z</v>
+        <v>2022-05-08T00:00:00.000Z</v>
       </c>
       <c r="H50">
         <v>58700</v>
@@ -2170,7 +2170,7 @@
         <v>22</v>
       </c>
       <c r="G51" s="1" t="d">
-        <v>2022-04-06T05:30:00.000Z</v>
+        <v>2022-04-06T00:00:00.000Z</v>
       </c>
       <c r="H51">
         <v>51500</v>
@@ -2205,7 +2205,7 @@
         <v>54</v>
       </c>
       <c r="G52" s="1" t="d">
-        <v>2025-07-27T05:30:00.000Z</v>
+        <v>2025-07-27T00:00:00.000Z</v>
       </c>
       <c r="H52">
         <v>64900</v>
@@ -2240,7 +2240,7 @@
         <v>24</v>
       </c>
       <c r="G53" s="1" t="d">
-        <v>2016-09-28T05:30:00.000Z</v>
+        <v>2016-09-28T00:00:00.000Z</v>
       </c>
       <c r="H53">
         <v>73200</v>
@@ -2275,7 +2275,7 @@
         <v>27</v>
       </c>
       <c r="G54" s="1" t="d">
-        <v>2016-12-13T05:30:00.000Z</v>
+        <v>2016-12-13T00:00:00.000Z</v>
       </c>
       <c r="H54">
         <v>43800</v>
@@ -2310,7 +2310,7 @@
         <v>56</v>
       </c>
       <c r="G55" s="1" t="d">
-        <v>2020-03-15T05:30:00.000Z</v>
+        <v>2020-03-15T00:00:00.000Z</v>
       </c>
       <c r="H55">
         <v>56700</v>
@@ -2345,7 +2345,7 @@
         <v>52</v>
       </c>
       <c r="G56" s="1" t="d">
-        <v>2023-05-28T05:30:00.000Z</v>
+        <v>2023-05-28T00:00:00.000Z</v>
       </c>
       <c r="H56">
         <v>46900</v>
@@ -2380,7 +2380,7 @@
         <v>28</v>
       </c>
       <c r="G57" s="1" t="d">
-        <v>2018-08-24T05:30:00.000Z</v>
+        <v>2018-08-24T00:00:00.000Z</v>
       </c>
       <c r="H57">
         <v>73600</v>
@@ -2415,7 +2415,7 @@
         <v>58</v>
       </c>
       <c r="G58" s="1" t="d">
-        <v>2018-04-15T05:30:00.000Z</v>
+        <v>2018-04-15T00:00:00.000Z</v>
       </c>
       <c r="H58">
         <v>47000</v>
@@ -2450,7 +2450,7 @@
         <v>49</v>
       </c>
       <c r="G59" s="1" t="d">
-        <v>2017-07-18T05:30:00.000Z</v>
+        <v>2017-07-18T00:00:00.000Z</v>
       </c>
       <c r="H59">
         <v>66100</v>
@@ -2485,7 +2485,7 @@
         <v>39</v>
       </c>
       <c r="G60" s="1" t="d">
-        <v>2025-09-21T05:30:00.000Z</v>
+        <v>2025-09-21T00:00:00.000Z</v>
       </c>
       <c r="H60">
         <v>53300</v>
@@ -2520,7 +2520,7 @@
         <v>41</v>
       </c>
       <c r="G61" s="1" t="d">
-        <v>2018-05-04T05:30:00.000Z</v>
+        <v>2018-05-04T00:00:00.000Z</v>
       </c>
       <c r="H61">
         <v>85000</v>
@@ -2555,7 +2555,7 @@
         <v>51</v>
       </c>
       <c r="G62" s="1" t="d">
-        <v>2025-03-04T05:30:00.000Z</v>
+        <v>2025-03-04T00:00:00.000Z</v>
       </c>
       <c r="H62">
         <v>34500</v>
@@ -2590,7 +2590,7 @@
         <v>49</v>
       </c>
       <c r="G63" s="1" t="d">
-        <v>2024-12-09T05:30:00.000Z</v>
+        <v>2024-12-09T00:00:00.000Z</v>
       </c>
       <c r="H63">
         <v>40600</v>
@@ -2625,7 +2625,7 @@
         <v>27</v>
       </c>
       <c r="G64" s="1" t="d">
-        <v>2017-01-28T05:30:00.000Z</v>
+        <v>2017-01-28T00:00:00.000Z</v>
       </c>
       <c r="H64">
         <v>37800</v>
@@ -2660,7 +2660,7 @@
         <v>43</v>
       </c>
       <c r="G65" s="1" t="d">
-        <v>2023-05-17T05:30:00.000Z</v>
+        <v>2023-05-17T00:00:00.000Z</v>
       </c>
       <c r="H65">
         <v>42000</v>
@@ -2695,7 +2695,7 @@
         <v>56</v>
       </c>
       <c r="G66" s="1" t="d">
-        <v>2022-02-09T05:30:00.000Z</v>
+        <v>2022-02-09T00:00:00.000Z</v>
       </c>
       <c r="H66">
         <v>70900</v>
@@ -2730,7 +2730,7 @@
         <v>53</v>
       </c>
       <c r="G67" s="1" t="d">
-        <v>2024-04-25T05:30:00.000Z</v>
+        <v>2024-04-25T00:00:00.000Z</v>
       </c>
       <c r="H67">
         <v>54100</v>
@@ -2765,7 +2765,7 @@
         <v>34</v>
       </c>
       <c r="G68" s="1" t="d">
-        <v>2018-06-25T05:30:00.000Z</v>
+        <v>2018-06-25T00:00:00.000Z</v>
       </c>
       <c r="H68">
         <v>75600</v>
@@ -2800,7 +2800,7 @@
         <v>45</v>
       </c>
       <c r="G69" s="1" t="d">
-        <v>2023-12-24T05:30:00.000Z</v>
+        <v>2023-12-24T00:00:00.000Z</v>
       </c>
       <c r="H69">
         <v>65900</v>
@@ -2835,7 +2835,7 @@
         <v>49</v>
       </c>
       <c r="G70" s="1" t="d">
-        <v>2021-11-09T05:30:00.000Z</v>
+        <v>2021-11-09T00:00:00.000Z</v>
       </c>
       <c r="H70">
         <v>57100</v>
@@ -2870,7 +2870,7 @@
         <v>43</v>
       </c>
       <c r="G71" s="1" t="d">
-        <v>2024-08-23T05:30:00.000Z</v>
+        <v>2024-08-23T00:00:00.000Z</v>
       </c>
       <c r="H71">
         <v>45200</v>
@@ -2905,7 +2905,7 @@
         <v>54</v>
       </c>
       <c r="G72" s="1" t="d">
-        <v>2024-06-26T05:30:00.000Z</v>
+        <v>2024-06-26T00:00:00.000Z</v>
       </c>
       <c r="H72">
         <v>52400</v>
@@ -2940,7 +2940,7 @@
         <v>57</v>
       </c>
       <c r="G73" s="1" t="d">
-        <v>2016-03-06T05:30:00.000Z</v>
+        <v>2016-03-06T00:00:00.000Z</v>
       </c>
       <c r="H73">
         <v>109300</v>
@@ -2975,7 +2975,7 @@
         <v>50</v>
       </c>
       <c r="G74" s="1" t="d">
-        <v>2016-10-10T05:30:00.000Z</v>
+        <v>2016-10-10T00:00:00.000Z</v>
       </c>
       <c r="H74">
         <v>95800</v>
@@ -3010,7 +3010,7 @@
         <v>24</v>
       </c>
       <c r="G75" s="1" t="d">
-        <v>2023-05-09T05:30:00.000Z</v>
+        <v>2023-05-09T00:00:00.000Z</v>
       </c>
       <c r="H75">
         <v>52000</v>
@@ -3045,7 +3045,7 @@
         <v>40</v>
       </c>
       <c r="G76" s="1" t="d">
-        <v>2021-09-21T05:30:00.000Z</v>
+        <v>2021-09-21T00:00:00.000Z</v>
       </c>
       <c r="H76">
         <v>73800</v>
@@ -3080,7 +3080,7 @@
         <v>51</v>
       </c>
       <c r="G77" s="1" t="d">
-        <v>2025-02-11T05:30:00.000Z</v>
+        <v>2025-02-11T00:00:00.000Z</v>
       </c>
       <c r="H77">
         <v>34800</v>
@@ -3115,7 +3115,7 @@
         <v>25</v>
       </c>
       <c r="G78" s="1" t="d">
-        <v>2024-03-15T05:30:00.000Z</v>
+        <v>2024-03-15T00:00:00.000Z</v>
       </c>
       <c r="H78">
         <v>81100</v>
@@ -3150,7 +3150,7 @@
         <v>42</v>
       </c>
       <c r="G79" s="1" t="d">
-        <v>2025-12-23T05:30:00.000Z</v>
+        <v>2025-12-23T00:00:00.000Z</v>
       </c>
       <c r="H79">
         <v>73200</v>
@@ -3185,7 +3185,7 @@
         <v>31</v>
       </c>
       <c r="G80" s="1" t="d">
-        <v>2016-01-28T05:30:00.000Z</v>
+        <v>2016-01-28T00:00:00.000Z</v>
       </c>
       <c r="H80">
         <v>47100</v>
@@ -3220,7 +3220,7 @@
         <v>35</v>
       </c>
       <c r="G81" s="1" t="d">
-        <v>2020-09-11T05:30:00.000Z</v>
+        <v>2020-09-11T00:00:00.000Z</v>
       </c>
       <c r="H81">
         <v>79700</v>
@@ -3255,7 +3255,7 @@
         <v>38</v>
       </c>
       <c r="G82" s="1" t="d">
-        <v>2021-04-06T05:30:00.000Z</v>
+        <v>2021-04-06T00:00:00.000Z</v>
       </c>
       <c r="H82">
         <v>57600</v>
@@ -3290,7 +3290,7 @@
         <v>40</v>
       </c>
       <c r="G83" s="1" t="d">
-        <v>2020-07-03T05:30:00.000Z</v>
+        <v>2020-07-03T00:00:00.000Z</v>
       </c>
       <c r="H83">
         <v>97000</v>
@@ -3325,7 +3325,7 @@
         <v>54</v>
       </c>
       <c r="G84" s="1" t="d">
-        <v>2022-10-11T05:30:00.000Z</v>
+        <v>2022-10-11T00:00:00.000Z</v>
       </c>
       <c r="H84">
         <v>126600</v>
@@ -3360,7 +3360,7 @@
         <v>44</v>
       </c>
       <c r="G85" s="1" t="d">
-        <v>2020-06-28T05:30:00.000Z</v>
+        <v>2020-06-28T00:00:00.000Z</v>
       </c>
       <c r="H85">
         <v>57300</v>
@@ -3395,7 +3395,7 @@
         <v>31</v>
       </c>
       <c r="G86" s="1" t="d">
-        <v>2021-01-04T05:30:00.000Z</v>
+        <v>2021-01-04T00:00:00.000Z</v>
       </c>
       <c r="H86">
         <v>56600</v>
@@ -3430,7 +3430,7 @@
         <v>31</v>
       </c>
       <c r="G87" s="1" t="d">
-        <v>2025-08-15T05:30:00.000Z</v>
+        <v>2025-08-15T00:00:00.000Z</v>
       </c>
       <c r="H87">
         <v>53800</v>
@@ -3465,7 +3465,7 @@
         <v>53</v>
       </c>
       <c r="G88" s="1" t="d">
-        <v>2019-06-01T05:30:00.000Z</v>
+        <v>2019-06-01T00:00:00.000Z</v>
       </c>
       <c r="H88">
         <v>101300</v>
@@ -3500,7 +3500,7 @@
         <v>38</v>
       </c>
       <c r="G89" s="1" t="d">
-        <v>2020-03-26T05:30:00.000Z</v>
+        <v>2020-03-26T00:00:00.000Z</v>
       </c>
       <c r="H89">
         <v>94600</v>
@@ -3535,7 +3535,7 @@
         <v>40</v>
       </c>
       <c r="G90" s="1" t="d">
-        <v>2024-07-19T05:30:00.000Z</v>
+        <v>2024-07-19T00:00:00.000Z</v>
       </c>
       <c r="H90">
         <v>73700</v>
@@ -3570,7 +3570,7 @@
         <v>51</v>
       </c>
       <c r="G91" s="1" t="d">
-        <v>2019-07-22T05:30:00.000Z</v>
+        <v>2019-07-22T00:00:00.000Z</v>
       </c>
       <c r="H91">
         <v>47200</v>
@@ -3605,7 +3605,7 @@
         <v>50</v>
       </c>
       <c r="G92" s="1" t="d">
-        <v>2024-04-21T05:30:00.000Z</v>
+        <v>2024-04-21T00:00:00.000Z</v>
       </c>
       <c r="H92">
         <v>45700</v>
@@ -3640,7 +3640,7 @@
         <v>31</v>
       </c>
       <c r="G93" s="1" t="d">
-        <v>2020-07-26T05:30:00.000Z</v>
+        <v>2020-07-26T00:00:00.000Z</v>
       </c>
       <c r="H93">
         <v>47400</v>
@@ -3675,7 +3675,7 @@
         <v>28</v>
       </c>
       <c r="G94" s="1" t="d">
-        <v>2023-08-22T05:30:00.000Z</v>
+        <v>2023-08-22T00:00:00.000Z</v>
       </c>
       <c r="H94">
         <v>49100</v>
@@ -3710,7 +3710,7 @@
         <v>58</v>
       </c>
       <c r="G95" s="1" t="d">
-        <v>2021-10-28T05:30:00.000Z</v>
+        <v>2021-10-28T00:00:00.000Z</v>
       </c>
       <c r="H95">
         <v>32700</v>
@@ -3745,7 +3745,7 @@
         <v>37</v>
       </c>
       <c r="G96" s="1" t="d">
-        <v>2020-06-21T05:30:00.000Z</v>
+        <v>2020-06-21T00:00:00.000Z</v>
       </c>
       <c r="H96">
         <v>65900</v>
@@ -3780,7 +3780,7 @@
         <v>32</v>
       </c>
       <c r="G97" s="1" t="d">
-        <v>2022-06-22T05:30:00.000Z</v>
+        <v>2022-06-22T00:00:00.000Z</v>
       </c>
       <c r="H97">
         <v>59000</v>
@@ -3815,7 +3815,7 @@
         <v>53</v>
       </c>
       <c r="G98" s="1" t="d">
-        <v>2022-01-02T05:30:00.000Z</v>
+        <v>2022-01-02T00:00:00.000Z</v>
       </c>
       <c r="H98">
         <v>79800</v>
@@ -3850,7 +3850,7 @@
         <v>46</v>
       </c>
       <c r="G99" s="1" t="d">
-        <v>2025-02-06T05:30:00.000Z</v>
+        <v>2025-02-06T00:00:00.000Z</v>
       </c>
       <c r="H99">
         <v>131300</v>
@@ -3885,7 +3885,7 @@
         <v>37</v>
       </c>
       <c r="G100" s="1" t="d">
-        <v>2018-07-02T05:30:00.000Z</v>
+        <v>2018-07-02T00:00:00.000Z</v>
       </c>
       <c r="H100">
         <v>132800</v>
@@ -3920,7 +3920,7 @@
         <v>22</v>
       </c>
       <c r="G101" s="1" t="d">
-        <v>2025-08-12T05:30:00.000Z</v>
+        <v>2025-08-12T00:00:00.000Z</v>
       </c>
       <c r="H101">
         <v>56000</v>
@@ -3955,7 +3955,7 @@
         <v>31</v>
       </c>
       <c r="G102" s="1" t="d">
-        <v>2022-12-28T05:30:00.000Z</v>
+        <v>2022-12-28T00:00:00.000Z</v>
       </c>
       <c r="H102">
         <v>58700</v>
@@ -3990,7 +3990,7 @@
         <v>24</v>
       </c>
       <c r="G103" s="1" t="d">
-        <v>2020-12-11T05:30:00.000Z</v>
+        <v>2020-12-11T00:00:00.000Z</v>
       </c>
       <c r="H103">
         <v>52600</v>
@@ -4025,7 +4025,7 @@
         <v>46</v>
       </c>
       <c r="G104" s="1" t="d">
-        <v>2024-05-04T05:30:00.000Z</v>
+        <v>2024-05-04T00:00:00.000Z</v>
       </c>
       <c r="H104">
         <v>35900</v>
@@ -4060,7 +4060,7 @@
         <v>53</v>
       </c>
       <c r="G105" s="1" t="d">
-        <v>2016-06-17T05:30:00.000Z</v>
+        <v>2016-06-17T00:00:00.000Z</v>
       </c>
       <c r="H105">
         <v>70000</v>
@@ -4095,7 +4095,7 @@
         <v>33</v>
       </c>
       <c r="G106" s="1" t="d">
-        <v>2021-02-12T05:30:00.000Z</v>
+        <v>2021-02-12T00:00:00.000Z</v>
       </c>
       <c r="H106">
         <v>60000</v>
@@ -4130,7 +4130,7 @@
         <v>46</v>
       </c>
       <c r="G107" s="1" t="d">
-        <v>2020-01-16T05:30:00.000Z</v>
+        <v>2020-01-16T00:00:00.000Z</v>
       </c>
       <c r="H107">
         <v>52100</v>
@@ -4165,7 +4165,7 @@
         <v>42</v>
       </c>
       <c r="G108" s="1" t="d">
-        <v>2020-08-08T05:30:00.000Z</v>
+        <v>2020-08-08T00:00:00.000Z</v>
       </c>
       <c r="H108">
         <v>58300</v>
@@ -4200,7 +4200,7 @@
         <v>37</v>
       </c>
       <c r="G109" s="1" t="d">
-        <v>2017-05-09T05:30:00.000Z</v>
+        <v>2017-05-09T00:00:00.000Z</v>
       </c>
       <c r="H109">
         <v>61200</v>
@@ -4235,7 +4235,7 @@
         <v>49</v>
       </c>
       <c r="G110" s="1" t="d">
-        <v>2023-11-26T05:30:00.000Z</v>
+        <v>2023-11-26T00:00:00.000Z</v>
       </c>
       <c r="H110">
         <v>79900</v>
@@ -4270,7 +4270,7 @@
         <v>41</v>
       </c>
       <c r="G111" s="1" t="d">
-        <v>2019-02-02T05:30:00.000Z</v>
+        <v>2019-02-02T00:00:00.000Z</v>
       </c>
       <c r="H111">
         <v>124300</v>
@@ -4305,7 +4305,7 @@
         <v>26</v>
       </c>
       <c r="G112" s="1" t="d">
-        <v>2017-11-03T05:30:00.000Z</v>
+        <v>2017-11-03T00:00:00.000Z</v>
       </c>
       <c r="H112">
         <v>57100</v>
@@ -4340,7 +4340,7 @@
         <v>37</v>
       </c>
       <c r="G113" s="1" t="d">
-        <v>2024-08-20T05:30:00.000Z</v>
+        <v>2024-08-20T00:00:00.000Z</v>
       </c>
       <c r="H113">
         <v>94800</v>
@@ -4375,7 +4375,7 @@
         <v>36</v>
       </c>
       <c r="G114" s="1" t="d">
-        <v>2020-01-04T05:30:00.000Z</v>
+        <v>2020-01-04T00:00:00.000Z</v>
       </c>
       <c r="H114">
         <v>32200</v>
@@ -4410,7 +4410,7 @@
         <v>34</v>
       </c>
       <c r="G115" s="1" t="d">
-        <v>2018-03-05T05:30:00.000Z</v>
+        <v>2018-03-05T00:00:00.000Z</v>
       </c>
       <c r="H115">
         <v>59500</v>
@@ -4445,7 +4445,7 @@
         <v>26</v>
       </c>
       <c r="G116" s="1" t="d">
-        <v>2021-12-18T05:30:00.000Z</v>
+        <v>2021-12-18T00:00:00.000Z</v>
       </c>
       <c r="H116">
         <v>57500</v>
@@ -4480,7 +4480,7 @@
         <v>27</v>
       </c>
       <c r="G117" s="1" t="d">
-        <v>2017-03-18T05:30:00.000Z</v>
+        <v>2017-03-18T00:00:00.000Z</v>
       </c>
       <c r="H117">
         <v>70900</v>
@@ -4515,7 +4515,7 @@
         <v>47</v>
       </c>
       <c r="G118" s="1" t="d">
-        <v>2017-09-24T05:30:00.000Z</v>
+        <v>2017-09-24T00:00:00.000Z</v>
       </c>
       <c r="H118">
         <v>88000</v>
@@ -4550,7 +4550,7 @@
         <v>28</v>
       </c>
       <c r="G119" s="1" t="d">
-        <v>2018-02-15T05:30:00.000Z</v>
+        <v>2018-02-15T00:00:00.000Z</v>
       </c>
       <c r="H119">
         <v>60800</v>
@@ -4585,7 +4585,7 @@
         <v>27</v>
       </c>
       <c r="G120" s="1" t="d">
-        <v>2022-12-19T05:30:00.000Z</v>
+        <v>2022-12-19T00:00:00.000Z</v>
       </c>
       <c r="H120">
         <v>85300</v>
@@ -4620,7 +4620,7 @@
         <v>45</v>
       </c>
       <c r="G121" s="1" t="d">
-        <v>2019-04-05T05:30:00.000Z</v>
+        <v>2019-04-05T00:00:00.000Z</v>
       </c>
       <c r="H121">
         <v>95000</v>
@@ -4655,7 +4655,7 @@
         <v>58</v>
       </c>
       <c r="G122" s="1" t="d">
-        <v>2024-06-08T05:30:00.000Z</v>
+        <v>2024-06-08T00:00:00.000Z</v>
       </c>
       <c r="H122">
         <v>46500</v>
@@ -4690,7 +4690,7 @@
         <v>41</v>
       </c>
       <c r="G123" s="1" t="d">
-        <v>2022-11-24T05:30:00.000Z</v>
+        <v>2022-11-24T00:00:00.000Z</v>
       </c>
       <c r="H123">
         <v>61600</v>
@@ -4725,7 +4725,7 @@
         <v>22</v>
       </c>
       <c r="G124" s="1" t="d">
-        <v>2023-07-03T05:30:00.000Z</v>
+        <v>2023-07-03T00:00:00.000Z</v>
       </c>
       <c r="H124">
         <v>73200</v>
@@ -4760,7 +4760,7 @@
         <v>23</v>
       </c>
       <c r="G125" s="1" t="d">
-        <v>2024-12-24T05:30:00.000Z</v>
+        <v>2024-12-24T00:00:00.000Z</v>
       </c>
       <c r="H125">
         <v>99300</v>
@@ -4795,7 +4795,7 @@
         <v>45</v>
       </c>
       <c r="G126" s="1" t="d">
-        <v>2020-08-03T05:30:00.000Z</v>
+        <v>2020-08-03T00:00:00.000Z</v>
       </c>
       <c r="H126">
         <v>126800</v>
@@ -4830,7 +4830,7 @@
         <v>55</v>
       </c>
       <c r="G127" s="1" t="d">
-        <v>2018-12-05T05:30:00.000Z</v>
+        <v>2018-12-05T00:00:00.000Z</v>
       </c>
       <c r="H127">
         <v>95100</v>
@@ -4865,7 +4865,7 @@
         <v>56</v>
       </c>
       <c r="G128" s="1" t="d">
-        <v>2019-01-27T05:30:00.000Z</v>
+        <v>2019-01-27T00:00:00.000Z</v>
       </c>
       <c r="H128">
         <v>66200</v>
@@ -4900,7 +4900,7 @@
         <v>40</v>
       </c>
       <c r="G129" s="1" t="d">
-        <v>2020-06-09T05:30:00.000Z</v>
+        <v>2020-06-09T00:00:00.000Z</v>
       </c>
       <c r="H129">
         <v>77900</v>
@@ -4935,7 +4935,7 @@
         <v>34</v>
       </c>
       <c r="G130" s="1" t="d">
-        <v>2017-10-06T05:30:00.000Z</v>
+        <v>2017-10-06T00:00:00.000Z</v>
       </c>
       <c r="H130">
         <v>58500</v>
@@ -4970,7 +4970,7 @@
         <v>32</v>
       </c>
       <c r="G131" s="1" t="d">
-        <v>2018-12-17T05:30:00.000Z</v>
+        <v>2018-12-17T00:00:00.000Z</v>
       </c>
       <c r="H131">
         <v>71800</v>
@@ -5005,7 +5005,7 @@
         <v>49</v>
       </c>
       <c r="G132" s="1" t="d">
-        <v>2023-05-01T05:30:00.000Z</v>
+        <v>2023-05-01T00:00:00.000Z</v>
       </c>
       <c r="H132">
         <v>82000</v>
@@ -5040,7 +5040,7 @@
         <v>42</v>
       </c>
       <c r="G133" s="1" t="d">
-        <v>2019-04-02T05:30:00.000Z</v>
+        <v>2019-04-02T00:00:00.000Z</v>
       </c>
       <c r="H133">
         <v>65800</v>
@@ -5075,7 +5075,7 @@
         <v>44</v>
       </c>
       <c r="G134" s="1" t="d">
-        <v>2024-01-23T05:30:00.000Z</v>
+        <v>2024-01-23T00:00:00.000Z</v>
       </c>
       <c r="H134">
         <v>73500</v>
@@ -5110,7 +5110,7 @@
         <v>33</v>
       </c>
       <c r="G135" s="1" t="d">
-        <v>2024-12-21T05:30:00.000Z</v>
+        <v>2024-12-21T00:00:00.000Z</v>
       </c>
       <c r="H135">
         <v>68900</v>
@@ -5145,7 +5145,7 @@
         <v>40</v>
       </c>
       <c r="G136" s="1" t="d">
-        <v>2019-11-11T05:30:00.000Z</v>
+        <v>2019-11-11T00:00:00.000Z</v>
       </c>
       <c r="H136">
         <v>54800</v>
@@ -5180,7 +5180,7 @@
         <v>33</v>
       </c>
       <c r="G137" s="1" t="d">
-        <v>2025-03-16T05:30:00.000Z</v>
+        <v>2025-03-16T00:00:00.000Z</v>
       </c>
       <c r="H137">
         <v>57600</v>
@@ -5215,7 +5215,7 @@
         <v>49</v>
       </c>
       <c r="G138" s="1" t="d">
-        <v>2016-12-02T05:30:00.000Z</v>
+        <v>2016-12-02T00:00:00.000Z</v>
       </c>
       <c r="H138">
         <v>72100</v>
@@ -5250,7 +5250,7 @@
         <v>50</v>
       </c>
       <c r="G139" s="1" t="d">
-        <v>2018-06-14T05:30:00.000Z</v>
+        <v>2018-06-14T00:00:00.000Z</v>
       </c>
       <c r="H139">
         <v>36800</v>
@@ -5285,7 +5285,7 @@
         <v>40</v>
       </c>
       <c r="G140" s="1" t="d">
-        <v>2018-08-24T05:30:00.000Z</v>
+        <v>2018-08-24T00:00:00.000Z</v>
       </c>
       <c r="H140">
         <v>77400</v>
@@ -5320,7 +5320,7 @@
         <v>32</v>
       </c>
       <c r="G141" s="1" t="d">
-        <v>2019-05-26T05:30:00.000Z</v>
+        <v>2019-05-26T00:00:00.000Z</v>
       </c>
       <c r="H141">
         <v>75100</v>
@@ -5355,7 +5355,7 @@
         <v>52</v>
       </c>
       <c r="G142" s="1" t="d">
-        <v>2017-03-21T05:30:00.000Z</v>
+        <v>2017-03-21T00:00:00.000Z</v>
       </c>
       <c r="H142">
         <v>99000</v>
@@ -5390,7 +5390,7 @@
         <v>48</v>
       </c>
       <c r="G143" s="1" t="d">
-        <v>2018-07-20T05:30:00.000Z</v>
+        <v>2018-07-20T00:00:00.000Z</v>
       </c>
       <c r="H143">
         <v>95800</v>
@@ -5425,7 +5425,7 @@
         <v>55</v>
       </c>
       <c r="G144" s="1" t="d">
-        <v>2024-06-24T05:30:00.000Z</v>
+        <v>2024-06-24T00:00:00.000Z</v>
       </c>
       <c r="H144">
         <v>93800</v>
@@ -5460,7 +5460,7 @@
         <v>58</v>
       </c>
       <c r="G145" s="1" t="d">
-        <v>2017-06-13T05:30:00.000Z</v>
+        <v>2017-06-13T00:00:00.000Z</v>
       </c>
       <c r="H145">
         <v>79600</v>
@@ -5495,7 +5495,7 @@
         <v>52</v>
       </c>
       <c r="G146" s="1" t="d">
-        <v>2018-02-19T05:30:00.000Z</v>
+        <v>2018-02-19T00:00:00.000Z</v>
       </c>
       <c r="H146">
         <v>47800</v>
@@ -5530,7 +5530,7 @@
         <v>46</v>
       </c>
       <c r="G147" s="1" t="d">
-        <v>2019-07-25T05:30:00.000Z</v>
+        <v>2019-07-25T00:00:00.000Z</v>
       </c>
       <c r="H147">
         <v>56700</v>
@@ -5565,7 +5565,7 @@
         <v>55</v>
       </c>
       <c r="G148" s="1" t="d">
-        <v>2020-10-24T05:30:00.000Z</v>
+        <v>2020-10-24T00:00:00.000Z</v>
       </c>
       <c r="H148">
         <v>82300</v>
@@ -5600,7 +5600,7 @@
         <v>26</v>
       </c>
       <c r="G149" s="1" t="d">
-        <v>2022-09-16T05:30:00.000Z</v>
+        <v>2022-09-16T00:00:00.000Z</v>
       </c>
       <c r="H149">
         <v>74500</v>
@@ -5635,7 +5635,7 @@
         <v>58</v>
       </c>
       <c r="G150" s="1" t="d">
-        <v>2017-08-11T05:30:00.000Z</v>
+        <v>2017-08-11T00:00:00.000Z</v>
       </c>
       <c r="H150">
         <v>61500</v>
@@ -5670,7 +5670,7 @@
         <v>34</v>
       </c>
       <c r="G151" s="1" t="d">
-        <v>2024-07-11T05:30:00.000Z</v>
+        <v>2024-07-11T00:00:00.000Z</v>
       </c>
       <c r="H151">
         <v>50100</v>
@@ -5705,7 +5705,7 @@
         <v>37</v>
       </c>
       <c r="G152" s="1" t="d">
-        <v>2017-12-04T05:30:00.000Z</v>
+        <v>2017-12-04T00:00:00.000Z</v>
       </c>
       <c r="H152">
         <v>80200</v>
@@ -5740,7 +5740,7 @@
         <v>48</v>
       </c>
       <c r="G153" s="1" t="d">
-        <v>2018-10-07T05:30:00.000Z</v>
+        <v>2018-10-07T00:00:00.000Z</v>
       </c>
       <c r="H153">
         <v>76700</v>
@@ -5775,7 +5775,7 @@
         <v>28</v>
       </c>
       <c r="G154" s="1" t="d">
-        <v>2019-09-27T05:30:00.000Z</v>
+        <v>2019-09-27T00:00:00.000Z</v>
       </c>
       <c r="H154">
         <v>56700</v>
@@ -5810,7 +5810,7 @@
         <v>55</v>
       </c>
       <c r="G155" s="1" t="d">
-        <v>2022-01-03T05:30:00.000Z</v>
+        <v>2022-01-03T00:00:00.000Z</v>
       </c>
       <c r="H155">
         <v>129500</v>
@@ -5845,7 +5845,7 @@
         <v>22</v>
       </c>
       <c r="G156" s="1" t="d">
-        <v>2018-05-25T05:30:00.000Z</v>
+        <v>2018-05-25T00:00:00.000Z</v>
       </c>
       <c r="H156">
         <v>47200</v>
@@ -5880,7 +5880,7 @@
         <v>41</v>
       </c>
       <c r="G157" s="1" t="d">
-        <v>2022-12-25T05:30:00.000Z</v>
+        <v>2022-12-25T00:00:00.000Z</v>
       </c>
       <c r="H157">
         <v>83600</v>
@@ -5915,7 +5915,7 @@
         <v>24</v>
       </c>
       <c r="G158" s="1" t="d">
-        <v>2020-06-24T05:30:00.000Z</v>
+        <v>2020-06-24T00:00:00.000Z</v>
       </c>
       <c r="H158">
         <v>49300</v>
@@ -5950,7 +5950,7 @@
         <v>58</v>
       </c>
       <c r="G159" s="1" t="d">
-        <v>2021-08-28T05:30:00.000Z</v>
+        <v>2021-08-28T00:00:00.000Z</v>
       </c>
       <c r="H159">
         <v>40100</v>
@@ -5985,7 +5985,7 @@
         <v>52</v>
       </c>
       <c r="G160" s="1" t="d">
-        <v>2019-10-27T05:30:00.000Z</v>
+        <v>2019-10-27T00:00:00.000Z</v>
       </c>
       <c r="H160">
         <v>45100</v>
@@ -6020,7 +6020,7 @@
         <v>23</v>
       </c>
       <c r="G161" s="1" t="d">
-        <v>2021-01-10T05:30:00.000Z</v>
+        <v>2021-01-10T00:00:00.000Z</v>
       </c>
       <c r="H161">
         <v>31500</v>
@@ -6055,7 +6055,7 @@
         <v>50</v>
       </c>
       <c r="G162" s="1" t="d">
-        <v>2021-04-03T05:30:00.000Z</v>
+        <v>2021-04-03T00:00:00.000Z</v>
       </c>
       <c r="H162">
         <v>98100</v>
@@ -6090,7 +6090,7 @@
         <v>43</v>
       </c>
       <c r="G163" s="1" t="d">
-        <v>2022-06-04T05:30:00.000Z</v>
+        <v>2022-06-04T00:00:00.000Z</v>
       </c>
       <c r="H163">
         <v>31900</v>
@@ -6125,7 +6125,7 @@
         <v>36</v>
       </c>
       <c r="G164" s="1" t="d">
-        <v>2018-05-12T05:30:00.000Z</v>
+        <v>2018-05-12T00:00:00.000Z</v>
       </c>
       <c r="H164">
         <v>61500</v>
@@ -6160,7 +6160,7 @@
         <v>28</v>
       </c>
       <c r="G165" s="1" t="d">
-        <v>2023-05-06T05:30:00.000Z</v>
+        <v>2023-05-06T00:00:00.000Z</v>
       </c>
       <c r="H165">
         <v>120900</v>
@@ -6195,7 +6195,7 @@
         <v>45</v>
       </c>
       <c r="G166" s="1" t="d">
-        <v>2020-10-26T05:30:00.000Z</v>
+        <v>2020-10-26T00:00:00.000Z</v>
       </c>
       <c r="H166">
         <v>63400</v>
@@ -6230,7 +6230,7 @@
         <v>52</v>
       </c>
       <c r="G167" s="1" t="d">
-        <v>2025-04-13T05:30:00.000Z</v>
+        <v>2025-04-13T00:00:00.000Z</v>
       </c>
       <c r="H167">
         <v>66100</v>
@@ -6265,7 +6265,7 @@
         <v>43</v>
       </c>
       <c r="G168" s="1" t="d">
-        <v>2022-12-22T05:30:00.000Z</v>
+        <v>2022-12-22T00:00:00.000Z</v>
       </c>
       <c r="H168">
         <v>74900</v>
@@ -6300,7 +6300,7 @@
         <v>56</v>
       </c>
       <c r="G169" s="1" t="d">
-        <v>2018-07-20T05:30:00.000Z</v>
+        <v>2018-07-20T00:00:00.000Z</v>
       </c>
       <c r="H169">
         <v>67500</v>
@@ -6335,7 +6335,7 @@
         <v>53</v>
       </c>
       <c r="G170" s="1" t="d">
-        <v>2019-12-27T05:30:00.000Z</v>
+        <v>2019-12-27T00:00:00.000Z</v>
       </c>
       <c r="H170">
         <v>72600</v>
@@ -6370,7 +6370,7 @@
         <v>30</v>
       </c>
       <c r="G171" s="1" t="d">
-        <v>2018-11-02T05:30:00.000Z</v>
+        <v>2018-11-02T00:00:00.000Z</v>
       </c>
       <c r="H171">
         <v>99400</v>
@@ -6405,7 +6405,7 @@
         <v>32</v>
       </c>
       <c r="G172" s="1" t="d">
-        <v>2016-04-05T05:30:00.000Z</v>
+        <v>2016-04-05T00:00:00.000Z</v>
       </c>
       <c r="H172">
         <v>79100</v>
@@ -6440,7 +6440,7 @@
         <v>49</v>
       </c>
       <c r="G173" s="1" t="d">
-        <v>2017-05-08T05:30:00.000Z</v>
+        <v>2017-05-08T00:00:00.000Z</v>
       </c>
       <c r="H173">
         <v>42300</v>
@@ -6475,7 +6475,7 @@
         <v>53</v>
       </c>
       <c r="G174" s="1" t="d">
-        <v>2016-07-10T05:30:00.000Z</v>
+        <v>2016-07-10T00:00:00.000Z</v>
       </c>
       <c r="H174">
         <v>93100</v>
@@ -6510,7 +6510,7 @@
         <v>48</v>
       </c>
       <c r="G175" s="1" t="d">
-        <v>2025-04-22T05:30:00.000Z</v>
+        <v>2025-04-22T00:00:00.000Z</v>
       </c>
       <c r="H175">
         <v>56100</v>
@@ -6545,7 +6545,7 @@
         <v>39</v>
       </c>
       <c r="G176" s="1" t="d">
-        <v>2016-08-24T05:30:00.000Z</v>
+        <v>2016-08-24T00:00:00.000Z</v>
       </c>
       <c r="H176">
         <v>56100</v>
@@ -6580,7 +6580,7 @@
         <v>47</v>
       </c>
       <c r="G177" s="1" t="d">
-        <v>2021-07-28T05:30:00.000Z</v>
+        <v>2021-07-28T00:00:00.000Z</v>
       </c>
       <c r="H177">
         <v>50700</v>
@@ -6615,7 +6615,7 @@
         <v>39</v>
       </c>
       <c r="G178" s="1" t="d">
-        <v>2020-09-12T05:30:00.000Z</v>
+        <v>2020-09-12T00:00:00.000Z</v>
       </c>
       <c r="H178">
         <v>73500</v>
@@ -6650,7 +6650,7 @@
         <v>43</v>
       </c>
       <c r="G179" s="1" t="d">
-        <v>2019-11-10T05:30:00.000Z</v>
+        <v>2019-11-10T00:00:00.000Z</v>
       </c>
       <c r="H179">
         <v>84000</v>
@@ -6685,7 +6685,7 @@
         <v>43</v>
       </c>
       <c r="G180" s="1" t="d">
-        <v>2025-10-13T05:30:00.000Z</v>
+        <v>2025-10-13T00:00:00.000Z</v>
       </c>
       <c r="H180">
         <v>86000</v>
@@ -6720,7 +6720,7 @@
         <v>39</v>
       </c>
       <c r="G181" s="1" t="d">
-        <v>2019-09-16T05:30:00.000Z</v>
+        <v>2019-09-16T00:00:00.000Z</v>
       </c>
       <c r="H181">
         <v>81400</v>
@@ -6755,7 +6755,7 @@
         <v>54</v>
       </c>
       <c r="G182" s="1" t="d">
-        <v>2020-11-24T05:30:00.000Z</v>
+        <v>2020-11-24T00:00:00.000Z</v>
       </c>
       <c r="H182">
         <v>92800</v>
@@ -6790,7 +6790,7 @@
         <v>43</v>
       </c>
       <c r="G183" s="1" t="d">
-        <v>2024-02-20T05:30:00.000Z</v>
+        <v>2024-02-20T00:00:00.000Z</v>
       </c>
       <c r="H183">
         <v>52600</v>
@@ -6825,7 +6825,7 @@
         <v>52</v>
       </c>
       <c r="G184" s="1" t="d">
-        <v>2024-07-01T05:30:00.000Z</v>
+        <v>2024-07-01T00:00:00.000Z</v>
       </c>
       <c r="H184">
         <v>110100</v>
@@ -6860,7 +6860,7 @@
         <v>39</v>
       </c>
       <c r="G185" s="1" t="d">
-        <v>2023-09-06T05:30:00.000Z</v>
+        <v>2023-09-06T00:00:00.000Z</v>
       </c>
       <c r="H185">
         <v>71700</v>
@@ -6895,7 +6895,7 @@
         <v>34</v>
       </c>
       <c r="G186" s="1" t="d">
-        <v>2017-01-01T05:30:00.000Z</v>
+        <v>2017-01-01T00:00:00.000Z</v>
       </c>
       <c r="H186">
         <v>98300</v>
@@ -6930,7 +6930,7 @@
         <v>32</v>
       </c>
       <c r="G187" s="1" t="d">
-        <v>2023-04-21T05:30:00.000Z</v>
+        <v>2023-04-21T00:00:00.000Z</v>
       </c>
       <c r="H187">
         <v>57400</v>
@@ -6965,7 +6965,7 @@
         <v>32</v>
       </c>
       <c r="G188" s="1" t="d">
-        <v>2023-10-27T05:30:00.000Z</v>
+        <v>2023-10-27T00:00:00.000Z</v>
       </c>
       <c r="H188">
         <v>42400</v>
@@ -7000,7 +7000,7 @@
         <v>35</v>
       </c>
       <c r="G189" s="1" t="d">
-        <v>2021-04-20T05:30:00.000Z</v>
+        <v>2021-04-20T00:00:00.000Z</v>
       </c>
       <c r="H189">
         <v>63700</v>
@@ -7035,7 +7035,7 @@
         <v>25</v>
       </c>
       <c r="G190" s="1" t="d">
-        <v>2021-08-15T05:30:00.000Z</v>
+        <v>2021-08-15T00:00:00.000Z</v>
       </c>
       <c r="H190">
         <v>98400</v>
@@ -7070,7 +7070,7 @@
         <v>37</v>
       </c>
       <c r="G191" s="1" t="d">
-        <v>2020-07-25T05:30:00.000Z</v>
+        <v>2020-07-25T00:00:00.000Z</v>
       </c>
       <c r="H191">
         <v>40400</v>
@@ -7105,7 +7105,7 @@
         <v>25</v>
       </c>
       <c r="G192" s="1" t="d">
-        <v>2021-09-05T05:30:00.000Z</v>
+        <v>2021-09-05T00:00:00.000Z</v>
       </c>
       <c r="H192">
         <v>80600</v>
@@ -7140,7 +7140,7 @@
         <v>55</v>
       </c>
       <c r="G193" s="1" t="d">
-        <v>2017-10-25T05:30:00.000Z</v>
+        <v>2017-10-25T00:00:00.000Z</v>
       </c>
       <c r="H193">
         <v>43500</v>
@@ -7175,7 +7175,7 @@
         <v>44</v>
       </c>
       <c r="G194" s="1" t="d">
-        <v>2023-04-07T05:30:00.000Z</v>
+        <v>2023-04-07T00:00:00.000Z</v>
       </c>
       <c r="H194">
         <v>133500</v>
@@ -7210,7 +7210,7 @@
         <v>34</v>
       </c>
       <c r="G195" s="1" t="d">
-        <v>2018-01-11T05:30:00.000Z</v>
+        <v>2018-01-11T00:00:00.000Z</v>
       </c>
       <c r="H195">
         <v>80700</v>
@@ -7245,7 +7245,7 @@
         <v>43</v>
       </c>
       <c r="G196" s="1" t="d">
-        <v>2024-03-28T05:30:00.000Z</v>
+        <v>2024-03-28T00:00:00.000Z</v>
       </c>
       <c r="H196">
         <v>84000</v>
@@ -7280,7 +7280,7 @@
         <v>34</v>
       </c>
       <c r="G197" s="1" t="d">
-        <v>2025-07-15T05:30:00.000Z</v>
+        <v>2025-07-15T00:00:00.000Z</v>
       </c>
       <c r="H197">
         <v>55500</v>
@@ -7315,7 +7315,7 @@
         <v>40</v>
       </c>
       <c r="G198" s="1" t="d">
-        <v>2021-10-28T05:30:00.000Z</v>
+        <v>2021-10-28T00:00:00.000Z</v>
       </c>
       <c r="H198">
         <v>57200</v>
@@ -7350,7 +7350,7 @@
         <v>32</v>
       </c>
       <c r="G199" s="1" t="d">
-        <v>2021-12-21T05:30:00.000Z</v>
+        <v>2021-12-21T00:00:00.000Z</v>
       </c>
       <c r="H199">
         <v>82300</v>
@@ -7385,7 +7385,7 @@
         <v>39</v>
       </c>
       <c r="G200" s="1" t="d">
-        <v>2019-10-02T05:30:00.000Z</v>
+        <v>2019-10-02T00:00:00.000Z</v>
       </c>
       <c r="H200">
         <v>75900</v>
@@ -7420,7 +7420,7 @@
         <v>30</v>
       </c>
       <c r="G201" s="1" t="d">
-        <v>2016-01-05T05:30:00.000Z</v>
+        <v>2016-01-05T00:00:00.000Z</v>
       </c>
       <c r="H201">
         <v>84400</v>
@@ -7455,7 +7455,7 @@
         <v>54</v>
       </c>
       <c r="G202" s="1" t="d">
-        <v>2025-09-14T05:30:00.000Z</v>
+        <v>2025-09-14T00:00:00.000Z</v>
       </c>
       <c r="H202">
         <v>119300</v>
@@ -7490,7 +7490,7 @@
         <v>38</v>
       </c>
       <c r="G203" s="1" t="d">
-        <v>2021-08-10T05:30:00.000Z</v>
+        <v>2021-08-10T00:00:00.000Z</v>
       </c>
       <c r="H203">
         <v>44600</v>
@@ -7525,7 +7525,7 @@
         <v>37</v>
       </c>
       <c r="G204" s="1" t="d">
-        <v>2019-05-19T05:30:00.000Z</v>
+        <v>2019-05-19T00:00:00.000Z</v>
       </c>
       <c r="H204">
         <v>47500</v>
@@ -7560,7 +7560,7 @@
         <v>33</v>
       </c>
       <c r="G205" s="1" t="d">
-        <v>2023-03-05T05:30:00.000Z</v>
+        <v>2023-03-05T00:00:00.000Z</v>
       </c>
       <c r="H205">
         <v>41800</v>
@@ -7595,7 +7595,7 @@
         <v>24</v>
       </c>
       <c r="G206" s="1" t="d">
-        <v>2019-05-02T05:30:00.000Z</v>
+        <v>2019-05-02T00:00:00.000Z</v>
       </c>
       <c r="H206">
         <v>78500</v>
@@ -7630,7 +7630,7 @@
         <v>51</v>
       </c>
       <c r="G207" s="1" t="d">
-        <v>2020-03-16T05:30:00.000Z</v>
+        <v>2020-03-16T00:00:00.000Z</v>
       </c>
       <c r="H207">
         <v>103600</v>
@@ -7665,7 +7665,7 @@
         <v>41</v>
       </c>
       <c r="G208" s="1" t="d">
-        <v>2019-02-20T05:30:00.000Z</v>
+        <v>2019-02-20T00:00:00.000Z</v>
       </c>
       <c r="H208">
         <v>72800</v>
@@ -7700,7 +7700,7 @@
         <v>41</v>
       </c>
       <c r="G209" s="1" t="d">
-        <v>2024-01-15T05:30:00.000Z</v>
+        <v>2024-01-15T00:00:00.000Z</v>
       </c>
       <c r="H209">
         <v>90800</v>
@@ -7735,7 +7735,7 @@
         <v>57</v>
       </c>
       <c r="G210" s="1" t="d">
-        <v>2017-07-07T05:30:00.000Z</v>
+        <v>2017-07-07T00:00:00.000Z</v>
       </c>
       <c r="H210">
         <v>81300</v>
@@ -7770,7 +7770,7 @@
         <v>25</v>
       </c>
       <c r="G211" s="1" t="d">
-        <v>2019-05-05T05:30:00.000Z</v>
+        <v>2019-05-05T00:00:00.000Z</v>
       </c>
       <c r="H211">
         <v>79900</v>
@@ -7805,7 +7805,7 @@
         <v>48</v>
       </c>
       <c r="G212" s="1" t="d">
-        <v>2017-06-05T05:30:00.000Z</v>
+        <v>2017-06-05T00:00:00.000Z</v>
       </c>
       <c r="H212">
         <v>50000</v>
@@ -7840,7 +7840,7 @@
         <v>48</v>
       </c>
       <c r="G213" s="1" t="d">
-        <v>2016-01-19T05:30:00.000Z</v>
+        <v>2016-01-19T00:00:00.000Z</v>
       </c>
       <c r="H213">
         <v>61200</v>
@@ -7875,7 +7875,7 @@
         <v>37</v>
       </c>
       <c r="G214" s="1" t="d">
-        <v>2024-01-24T05:30:00.000Z</v>
+        <v>2024-01-24T00:00:00.000Z</v>
       </c>
       <c r="H214">
         <v>86300</v>
@@ -7910,7 +7910,7 @@
         <v>57</v>
       </c>
       <c r="G215" s="1" t="d">
-        <v>2017-01-28T05:30:00.000Z</v>
+        <v>2017-01-28T00:00:00.000Z</v>
       </c>
       <c r="H215">
         <v>69000</v>
@@ -7945,7 +7945,7 @@
         <v>51</v>
       </c>
       <c r="G216" s="1" t="d">
-        <v>2024-12-15T05:30:00.000Z</v>
+        <v>2024-12-15T00:00:00.000Z</v>
       </c>
       <c r="H216">
         <v>66800</v>
@@ -7980,7 +7980,7 @@
         <v>42</v>
       </c>
       <c r="G217" s="1" t="d">
-        <v>2022-06-20T05:30:00.000Z</v>
+        <v>2022-06-20T00:00:00.000Z</v>
       </c>
       <c r="H217">
         <v>54500</v>
@@ -8015,7 +8015,7 @@
         <v>30</v>
       </c>
       <c r="G218" s="1" t="d">
-        <v>2018-08-10T05:30:00.000Z</v>
+        <v>2018-08-10T00:00:00.000Z</v>
       </c>
       <c r="H218">
         <v>60700</v>
@@ -8050,7 +8050,7 @@
         <v>40</v>
       </c>
       <c r="G219" s="1" t="d">
-        <v>2016-01-04T05:30:00.000Z</v>
+        <v>2016-01-04T00:00:00.000Z</v>
       </c>
       <c r="H219">
         <v>81300</v>
@@ -8085,7 +8085,7 @@
         <v>56</v>
       </c>
       <c r="G220" s="1" t="d">
-        <v>2023-08-23T05:30:00.000Z</v>
+        <v>2023-08-23T00:00:00.000Z</v>
       </c>
       <c r="H220">
         <v>53800</v>
@@ -8120,7 +8120,7 @@
         <v>31</v>
       </c>
       <c r="G221" s="1" t="d">
-        <v>2021-04-21T05:30:00.000Z</v>
+        <v>2021-04-21T00:00:00.000Z</v>
       </c>
       <c r="H221">
         <v>61700</v>
@@ -8155,7 +8155,7 @@
         <v>26</v>
       </c>
       <c r="G222" s="1" t="d">
-        <v>2022-04-17T05:30:00.000Z</v>
+        <v>2022-04-17T00:00:00.000Z</v>
       </c>
       <c r="H222">
         <v>78700</v>
@@ -8190,7 +8190,7 @@
         <v>27</v>
       </c>
       <c r="G223" s="1" t="d">
-        <v>2024-12-15T05:30:00.000Z</v>
+        <v>2024-12-15T00:00:00.000Z</v>
       </c>
       <c r="H223">
         <v>77900</v>
@@ -8225,7 +8225,7 @@
         <v>46</v>
       </c>
       <c r="G224" s="1" t="d">
-        <v>2017-01-27T05:30:00.000Z</v>
+        <v>2017-01-27T00:00:00.000Z</v>
       </c>
       <c r="H224">
         <v>53900</v>
@@ -8260,7 +8260,7 @@
         <v>40</v>
       </c>
       <c r="G225" s="1" t="d">
-        <v>2018-10-26T05:30:00.000Z</v>
+        <v>2018-10-26T00:00:00.000Z</v>
       </c>
       <c r="H225">
         <v>55100</v>
@@ -8295,7 +8295,7 @@
         <v>33</v>
       </c>
       <c r="G226" s="1" t="d">
-        <v>2019-03-09T05:30:00.000Z</v>
+        <v>2019-03-09T00:00:00.000Z</v>
       </c>
       <c r="H226">
         <v>39100</v>
@@ -8330,7 +8330,7 @@
         <v>33</v>
       </c>
       <c r="G227" s="1" t="d">
-        <v>2022-02-16T05:30:00.000Z</v>
+        <v>2022-02-16T00:00:00.000Z</v>
       </c>
       <c r="H227">
         <v>134900</v>
@@ -8365,7 +8365,7 @@
         <v>46</v>
       </c>
       <c r="G228" s="1" t="d">
-        <v>2017-12-25T05:30:00.000Z</v>
+        <v>2017-12-25T00:00:00.000Z</v>
       </c>
       <c r="H228">
         <v>34600</v>
@@ -8400,7 +8400,7 @@
         <v>27</v>
       </c>
       <c r="G229" s="1" t="d">
-        <v>2024-04-27T05:30:00.000Z</v>
+        <v>2024-04-27T00:00:00.000Z</v>
       </c>
       <c r="H229">
         <v>55600</v>
@@ -8435,7 +8435,7 @@
         <v>44</v>
       </c>
       <c r="G230" s="1" t="d">
-        <v>2025-08-28T05:30:00.000Z</v>
+        <v>2025-08-28T00:00:00.000Z</v>
       </c>
       <c r="H230">
         <v>67000</v>
@@ -8470,7 +8470,7 @@
         <v>43</v>
       </c>
       <c r="G231" s="1" t="d">
-        <v>2017-01-23T05:30:00.000Z</v>
+        <v>2017-01-23T00:00:00.000Z</v>
       </c>
       <c r="H231">
         <v>55500</v>

</xml_diff>